<commit_message>
- Updated import Excel instructions for ## Step 5: Create new SharePoint site in docs\recruit-nextgen\00-course-setup\index.md - Added images to reflect the 3 new steps in ## Step 5: Create new SharePoint site - Renamed image files
</commit_message>
<xml_diff>
--- a/docs/recruit-nextgen/00-course-setup/assets/employee-assets/EmployeeAssets.xlsx
+++ b/docs/recruit-nextgen/00-course-setup/assets/employee-assets/EmployeeAssets.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://microsoftapc-my.sharepoint.com/personal/ebenitez_microsoft_com/Documents/Power Platform CA/Copilot Studio/Recruit V2/02_BuildADeclarativeAgent/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://microsoftapc-my.sharepoint.com/personal/ebenitez_microsoft_com/Documents/Power Platform CA/Copilot Studio/Recruit V2/00_CourseSetup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{97A8220B-E57D-4089-9ACD-21AEA2197D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40882172-CCB5-4D19-BD40-474F52F5531D}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{97A8220B-E57D-4089-9ACD-21AEA2197D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{663E6774-A167-4CE9-9A27-3F2D9348D191}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4AF361D4-52E5-4608-A34E-E9FC9A9E465A}"/>
   </bookViews>
@@ -146,19 +146,19 @@
     <t>POAZEBWD</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/microsoft/agent-academy/refs/heads/main/docs/recruit/00-course-setup/images/device-images/Surface-Laptop-13.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/microsoft/agent-academy/refs/heads/main/docs/recruit/00-course-setup/images/device-images/Surface-Laptop-15.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/microsoft/agent-academy/refs/heads/main/docs/recruit/00-course-setup/images/device-images/Surface-Pro-12.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/microsoft/agent-academy/refs/heads/main/docs/recruit/00-course-setup/images/device-images/Surface-Studio.png</t>
-  </si>
-  <si>
     <t>Image</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/microsoft/agent-academy/refs/heads/main/docs/recruit-nextgen/00-course-setup/assets/device-images/Surface-Laptop-13.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/microsoft/agent-academy/refs/heads/main/docs/recruit-nextgen/00-course-setup/assets/device-images/Surface-Laptop-15.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/microsoft/agent-academy/refs/heads/main/docs/recruit-nextgen/00-course-setup/assets/device-images/Surface-Pro-12.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/microsoft/agent-academy/refs/heads/main/docs/recruit-nextgen/00-course-setup/assets/device-images/Surface-Studio.png</t>
   </si>
 </sst>
 </file>
@@ -258,10 +258,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -648,7 +644,7 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -683,7 +679,7 @@
         <v>17</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -718,7 +714,7 @@
         <v>21</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
@@ -753,7 +749,7 @@
         <v>27</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
@@ -788,7 +784,7 @@
         <v>34</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>